<commit_message>
chore: batch commit all local changes (H1-H10/I1-I2/G8-G14/A17/B60/D3 enhancements + tests + templates)
</commit_message>
<xml_diff>
--- a/backend/wp_templates/A/A17  重大事项概要程序表.xlsx
+++ b/backend/wp_templates/A/A17  重大事项概要程序表.xlsx
@@ -1,37 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2025年张娟\底稿修改\2024年致同通用审计程序及底稿模板\1.致同审计程序及底稿模板（2024年）\5.完成阶段（A1-A30）\2.总结程序（A11-A20 )\A17 重大事项概要\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C99908E-66D2-4C60-8007-CB7E427048C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="0" windowWidth="22980" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="60" yWindow="0" windowWidth="22980" windowHeight="12360" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="A17 重大事项概要程序表" sheetId="5" r:id="rId1"/>
-    <sheet name="GT_Custom" sheetId="4" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A17 重大事项概要程序表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GT_Custom" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
-    <externalReference r:id="rId4"/>
-    <externalReference r:id="rId5"/>
-    <externalReference r:id="rId6"/>
-    <externalReference r:id="rId7"/>
-    <externalReference r:id="rId8"/>
-    <externalReference r:id="rId9"/>
-    <externalReference r:id="rId10"/>
-    <externalReference r:id="rId11"/>
-    <externalReference r:id="rId12"/>
-    <externalReference r:id="rId13"/>
-    <externalReference r:id="rId14"/>
-    <externalReference r:id="rId15"/>
-    <externalReference r:id="rId16"/>
-    <externalReference r:id="rId17"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
   </externalReferences>
   <definedNames>
     <definedName name="AS2DocOpenMode" hidden="1">"AS2DocumentEdit"</definedName>
@@ -152,8 +145,6 @@
     <definedName name="OtherConditions">#REF!</definedName>
     <definedName name="Pre_tax_materiality">#REF!</definedName>
     <definedName name="Precision">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'A17 重大事项概要程序表'!$A$1:$H$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'A17 重大事项概要程序表'!$5:$5</definedName>
     <definedName name="PY_all_Equity">#REF!</definedName>
     <definedName name="PY_all_Income">#REF!</definedName>
     <definedName name="PY_all_RetEarn">#REF!</definedName>
@@ -312,624 +303,450 @@
     <definedName name="资产合计94期末">[14]企业表一!$F$14</definedName>
     <definedName name="资产合计95期初">[14]企业表一!$G$14</definedName>
     <definedName name="资产合计95期末">[14]企业表一!$H$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'A17 重大事项概要程序表'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'A17 重大事项概要程序表'!$A$1:$H$10</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
-  <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>Custom 1</t>
-  </si>
-  <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>Custom 2</t>
-  </si>
-  <si>
-    <t>C3</t>
-  </si>
-  <si>
-    <t>Custom 3</t>
-  </si>
-  <si>
-    <t>C4</t>
-  </si>
-  <si>
-    <t>Custom 4</t>
-  </si>
-  <si>
-    <t>C5</t>
-  </si>
-  <si>
-    <t>Custom 5</t>
-  </si>
-  <si>
-    <t>C6</t>
-  </si>
-  <si>
-    <t>Custom 6</t>
-  </si>
-  <si>
-    <t>C7</t>
-  </si>
-  <si>
-    <t>Custom 7</t>
-  </si>
-  <si>
-    <t>C8</t>
-  </si>
-  <si>
-    <t>Custom 8</t>
-  </si>
-  <si>
-    <t>致同会计师事务所</t>
-  </si>
-  <si>
-    <t>客户名称：</t>
-  </si>
-  <si>
-    <t>编制人：</t>
-  </si>
-  <si>
-    <t>序号</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>是否适用</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>执行情况说明</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>索引号</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>A17</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>A17-1</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>A17-3</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>A17-4</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>A17-2</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>A17-6</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>程序</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>重大事项概要程序表</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>日期：</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>汇总重大职业判断以及需合伙人关注事项，详细说明审计程序执行情况。</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>确定在审计过程中识别的重大职业判断以及需合伙人关注事项是否包括在重大事项概要汇总表中：
-（1）引起特别风险的事项；
-（2）已更正或未更正的错报；
-（3）值得关注的缺陷和其他控制缺陷；
-（4）重大职业判断；
-（5）业务咨询和意见分歧；
-（6）导致注册会计师难以实施必要审计程序的情形；
-（7）可能导致出具非无保留意见审计报告的事项；
-（8）独立性威胁或利益冲突。</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>索引号：</t>
-  </si>
-  <si>
-    <t>会计期间：201X年度</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>复核人：</t>
-  </si>
-  <si>
-    <t>页  次：</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>执行人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">对于咨询的重大会计或审计事项咨询，确定咨询报告是否包括在审计工作底稿中。 </t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>对于项目组的专业意见分歧，确认己经得到解决。并将解决方式、解决过程、解决结论等记录于工作底稿。</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-  <si>
-    <t>召开项目组总结会并将会议纪要记录于工作底稿。</t>
-    <phoneticPr fontId="36" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="34">
-    <numFmt numFmtId="8" formatCode="&quot;¥&quot;#,##0.00;[Red]&quot;¥&quot;\-#,##0.00"/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="_-#,##0_-;\(#,##0\);_-\ \ &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-#,##0.00_-;\(#,##0.00\);_-\ \ &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="mmm/dd/yyyy;_-\ &quot;N/A&quot;_-;_-\ &quot;-&quot;_-"/>
-    <numFmt numFmtId="179" formatCode="mmm/yyyy;_-\ &quot;N/A&quot;_-;_-\ &quot;-&quot;_-"/>
-    <numFmt numFmtId="180" formatCode="_-#,##0%_-;\(#,##0%\);_-\ &quot;-&quot;_-"/>
-    <numFmt numFmtId="181" formatCode="_-#,###,_-;\(#,###,\);_-\ \ &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="182" formatCode="_-#,###.00,_-;\(#,###.00,\);_-\ \ &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="183" formatCode="_-#0&quot;.&quot;0,_-;\(#0&quot;.&quot;0,\);_-\ \ &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="184" formatCode="_-#0&quot;.&quot;0000_-;\(#0&quot;.&quot;0000\);_-\ \ &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="185" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="186" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
-    <numFmt numFmtId="187" formatCode="&quot;\&quot;#,##0;[Red]&quot;\&quot;&quot;\&quot;\-#,##0"/>
-    <numFmt numFmtId="188" formatCode="&quot;\&quot;#,##0.00;[Red]&quot;\&quot;&quot;\&quot;\-#,##0.00"/>
-    <numFmt numFmtId="189" formatCode="&quot;\&quot;#,##0;&quot;\&quot;&quot;\&quot;\-#,##0"/>
-    <numFmt numFmtId="190" formatCode="0%_);\(0%\)"/>
-    <numFmt numFmtId="191" formatCode="0%;\(0%\)"/>
-    <numFmt numFmtId="192" formatCode="0.0%"/>
-    <numFmt numFmtId="193" formatCode="#,##0&quot; F&quot;_);\(#,##0&quot; F&quot;\)"/>
-    <numFmt numFmtId="194" formatCode="&quot;$&quot;#,##0;[Red]&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;\-#,##0"/>
-    <numFmt numFmtId="195" formatCode="#,##0.0_);\(#,##0.0\)"/>
-    <numFmt numFmtId="196" formatCode="hh:mm\ AM/PM_)"/>
-    <numFmt numFmtId="197" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="198" formatCode=";;;"/>
-    <numFmt numFmtId="199" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="200" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="201" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="202" formatCode="0.00000000000_);[Red]\(0.00000000000\)"/>
-    <numFmt numFmtId="203" formatCode="0.0000000"/>
-    <numFmt numFmtId="204" formatCode="0.000000"/>
-    <numFmt numFmtId="205" formatCode="0.00000000"/>
-    <numFmt numFmtId="206" formatCode="_ * #,##0_)\ _F_ ;_ * \(#,##0\)\ _F_ ;_ * &quot;-&quot;_)\ _F_ ;_ @_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="30">
+    <numFmt numFmtId="164" formatCode="_-#,##0_-;\(#,##0\);_-\ \ &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-#,##0.00_-;\(#,##0.00\);_-\ \ &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="mmm/dd/yyyy;_-\ &quot;N/A&quot;_-;_-\ &quot;-&quot;_-"/>
+    <numFmt numFmtId="167" formatCode="mmm/yyyy;_-\ &quot;N/A&quot;_-;_-\ &quot;-&quot;_-"/>
+    <numFmt numFmtId="168" formatCode="_-#,##0%_-;\(#,##0%\);_-\ &quot;-&quot;_-"/>
+    <numFmt numFmtId="169" formatCode="_-#,###,_-;\(#,###,\);_-\ \ &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="_-#,###.00,_-;\(#,###.00,\);_-\ \ &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="171" formatCode="_-#0&quot;.&quot;0,_-;\(#0&quot;.&quot;0,\);_-\ \ &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="172" formatCode="_-#0&quot;.&quot;0000_-;\(#0&quot;.&quot;0000\);_-\ \ &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="173" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="174" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
+    <numFmt numFmtId="175" formatCode="&quot;\&quot;#,##0;[Red]&quot;\&quot;&quot;\&quot;\-#,##0"/>
+    <numFmt numFmtId="176" formatCode="&quot;\&quot;#,##0.00;[Red]&quot;\&quot;&quot;\&quot;\-#,##0.00"/>
+    <numFmt numFmtId="177" formatCode="&quot;\&quot;#,##0;&quot;\&quot;&quot;\&quot;\-#,##0"/>
+    <numFmt numFmtId="178" formatCode="0%_);\(0%\)"/>
+    <numFmt numFmtId="179" formatCode="0%;\(0%\)"/>
+    <numFmt numFmtId="180" formatCode="0.0%"/>
+    <numFmt numFmtId="181" formatCode="#,##0&quot; F&quot;_);\(#,##0&quot; F&quot;\)"/>
+    <numFmt numFmtId="182" formatCode="&quot;$&quot;#,##0;[Red]&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;&quot;$&quot;\-#,##0"/>
+    <numFmt numFmtId="183" formatCode="#,##0.0_);\(#,##0.0\)"/>
+    <numFmt numFmtId="184" formatCode="hh:mm\ AM/PM_)"/>
+    <numFmt numFmtId="185" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="186" formatCode=";;;"/>
+    <numFmt numFmtId="187" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="188" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="189" formatCode="0.00000000000_);[Red]\(0.00000000000\)"/>
+    <numFmt numFmtId="190" formatCode="0.0000000"/>
+    <numFmt numFmtId="191" formatCode="0.000000"/>
+    <numFmt numFmtId="192" formatCode="0.00000000"/>
+    <numFmt numFmtId="193" formatCode="_ * #,##0_)\ _F_ ;_ * \(#,##0\)\ _F_ ;_ * &quot;-&quot;_)\ _F_ ;_ @_ "/>
   </numFmts>
   <fonts count="64">
     <font>
-      <sz val="12"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <sz val="12"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="12"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="10"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color indexed="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <color indexed="10"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <sz val="10"/>
       <u val="singleAccounting"/>
       <vertAlign val="subscript"/>
-      <sz val="10"/>
+    </font>
+    <font>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
     <font>
-      <i/>
-      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="8"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="9"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="20"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Helv"/>
+      <family val="2"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="MS Sans Serif"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="52"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="9"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color indexed="23"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color indexed="36"/>
+      <sz val="7.5"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="17"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="56"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="56"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="56"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color indexed="12"/>
+      <sz val="7.5"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="62"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="52"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="60"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Courier"/>
+      <family val="3"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="63"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Helv"/>
+      <family val="2"/>
+      <color indexed="10"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Cambria"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color indexed="56"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color indexed="8"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color indexed="10"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="20"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <name val="Helv"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="MS Sans Serif"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="52"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color indexed="23"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="7.5"/>
-      <color indexed="36"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="17"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color indexed="56"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color indexed="56"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="56"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="7.5"/>
-      <color indexed="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="62"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="52"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="60"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Courier"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="63"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color indexed="10"/>
-      <name val="Helv"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color indexed="56"/>
-      <name val="Cambria"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
       <sz val="9"/>
-      <name val="宋体"/>
-      <family val="2"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color indexed="8"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color indexed="8"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="13"/>
       <name val="Tms Rmn"/>
       <family val="1"/>
+      <sz val="13"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
       <name val="Tms Rmn"/>
       <family val="1"/>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
     <font>
-      <b/>
-      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="8"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="MS Sans Serif"/>
       <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="9"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="7"/>
       <name val="Small Fonts"/>
       <family val="2"/>
+      <sz val="7"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color indexed="8"/>
       <name val="MS Sans Serif"/>
       <family val="2"/>
+      <color indexed="8"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color indexed="16"/>
       <name val="Century Schoolbook"/>
       <family val="1"/>
+      <color indexed="16"/>
+      <sz val="8"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color indexed="8"/>
       <sz val="9"/>
-      <color indexed="8"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
       <name val="MS Sans Serif"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="12"/>
       <name val="MS Sans Serif"/>
       <family val="2"/>
+      <sz val="12"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Geneva"/>
       <family val="2"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="11"/>
       <name val="明朝"/>
       <family val="2"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="8"/>
       <name val="Century Schoolbook"/>
       <family val="1"/>
+      <sz val="8"/>
     </font>
     <font>
-      <u/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color indexed="12"/>
       <sz val="10"/>
-      <color indexed="12"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
+      <u val="single"/>
     </font>
     <font>
-      <sz val="11"/>
       <name val="蹈框"/>
       <charset val="134"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="ＭＳ Ｐゴシック"/>
+      <charset val="134"/>
+      <family val="2"/>
       <sz val="11"/>
-      <name val="ＭＳ Ｐゴシック"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
-      <sz val="12"/>
       <name val="바탕체"/>
       <family val="3"/>
+      <sz val="12"/>
     </font>
     <font>
-      <b/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <b val="1"/>
       <sz val="10"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="10"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color rgb="FFFF0000"/>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color indexed="10"/>
       <sz val="10"/>
-      <color indexed="10"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <b val="1"/>
       <sz val="12"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <b val="1"/>
       <sz val="14"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="31">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -1064,7 +881,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59996337778862885"/>
+        <fgColor theme="7" tint="0.5999633777886288"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1086,7 +903,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1319,584 +1136,683 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="174">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1">
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" applyProtection="0">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="181" fontId="7" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="182" fontId="7" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="183" fontId="7" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="184" fontId="7" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0"/>
     <xf numFmtId="3" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="185" fontId="14" fillId="0" borderId="2" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="186" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="173" fontId="14" fillId="0" borderId="2"/>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="3"/>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="4"/>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="38" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="14" fontId="21" fillId="23" borderId="5">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="0"/>
+    <xf numFmtId="38" fontId="20" fillId="22" borderId="0"/>
+    <xf numFmtId="14" fontId="21" fillId="23" borderId="5" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="8"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="10" fontId="20" fillId="24" borderId="9" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="187" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="188" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="3"/>
+    <xf numFmtId="10" fontId="20" fillId="24" borderId="9"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="10"/>
+    <xf numFmtId="175" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0"/>
-    <xf numFmtId="189" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="30" fillId="20" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="190" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="177" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="11"/>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="12"/>
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="3" fontId="31" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="13"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyProtection="1">
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="191" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="192" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="10" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="193" fontId="1" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyProtection="0">
+    <xf numFmtId="179" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="180" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="10" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="181" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="15" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="16">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="16" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="194" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="38" fontId="41" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="37" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="195" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="39" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="40" fontId="41" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="196" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="185" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="197" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="198" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0">
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="182" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="38" fontId="41" fillId="0" borderId="0"/>
+    <xf numFmtId="37" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="183" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="39" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="40" fontId="41" fillId="0" borderId="0"/>
+    <xf numFmtId="184" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="173" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="185" fontId="38" fillId="0" borderId="0"/>
+    <xf numFmtId="186" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="28" borderId="9"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="199" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="200" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="201" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="202" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="187" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="188" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="189" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="37" fontId="43" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="22" borderId="9"/>
-    <xf numFmtId="4" fontId="42" fillId="0" borderId="0">
+    <xf numFmtId="4" fontId="42" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="45" fillId="0" borderId="0">
+    <xf numFmtId="4" fontId="45" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="29" borderId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="29" borderId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="9">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="9" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="30" borderId="0" applyNumberFormat="0" applyFill="0">
+    <xf numFmtId="0" fontId="49" fillId="30" borderId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="51" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="4" fontId="52" fillId="0" borderId="0">
+    <xf numFmtId="9" fontId="51" fillId="0" borderId="0"/>
+    <xf numFmtId="4" fontId="52" fillId="0" borderId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="4" fontId="50" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="203" fontId="35" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="8" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="204" fontId="35" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="205" fontId="35" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="4" fontId="50" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="190" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="8" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="191" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="192" fontId="35" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0"/>
-    <xf numFmtId="200" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="206" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0">
+    <xf numFmtId="187" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="193" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="38" fontId="55" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="40" fontId="55" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="38" fontId="55" fillId="0" borderId="0"/>
+    <xf numFmtId="40" fontId="55" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="56" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <protection locked="0"/>
+  <cellXfs count="25">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="70" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="70">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="18" xfId="70" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="70">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" xfId="70" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="70">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="71" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="71" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="71" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="18" xfId="71" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="18" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" xfId="71" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="27" borderId="19" xfId="72" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="57" fillId="27" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="72">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="27" borderId="1" xfId="71" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="57" fillId="27" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="27" borderId="19" xfId="71" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="57" fillId="27" borderId="19" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" xfId="72" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="72">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" xfId="73" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="73">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="1" xfId="73" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="73">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="1" xfId="71" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="1" xfId="71" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="71">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" xfId="70" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="70">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" xfId="70" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="70">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="174">
-    <cellStyle name="?" xfId="74" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="?餡_x000c_k" xfId="75" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="?餡_x000c_k?_x000d_^" xfId="76" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="?餡_x000c_k?_x000d_^黇_x0001_??_x0007__x0001__x0001_" xfId="77" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="@_text" xfId="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="_2005审计报表及附注-中国建材股份模板（房屋）" xfId="78" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="_2006年年报审计PBC表-XXX" xfId="79" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="_2006年年报审计填报资料" xfId="80" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="_PBC审核提示" xfId="81" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="_宝丽华房地产20051231" xfId="82" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="_保证金-企业填写部分" xfId="83" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="_北新房屋2004年审-刘" xfId="84" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="_北新股份2005年审工作底稿" xfId="85" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="_北新建材关连交易基础表051230（10－12月版）更新稿" xfId="86" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="_北新建材-会计报表附注模版" xfId="87" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="_北新龙之星2004年审工作底稿" xfId="88" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="_北新物流2005底稿-刘" xfId="89" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="_北新置换memo" xfId="90" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="_存货结转测试" xfId="91" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="_存货数量与明细05.12" xfId="92" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="_动力厂2004年审工作底稿-刘" xfId="93" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="_分工" xfId="94" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="_工程施工项目现场审计提示" xfId="95" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="_关联交易" xfId="96" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="_关联交易、往来统计表" xfId="97" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="_科目核对表" xfId="98" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
-    <cellStyle name="_母PL" xfId="99" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
-    <cellStyle name="_人员分工备忘录" xfId="100" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
-    <cellStyle name="_审计所需资料清单－子公司" xfId="101" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="_长期借款－江阴" xfId="102" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="{Comma [0]}" xfId="2" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
-    <cellStyle name="{Comma}" xfId="3" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
-    <cellStyle name="{Date}" xfId="4" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="{Month}" xfId="5" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="{Percent}" xfId="6" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
-    <cellStyle name="{Thousand [0]}" xfId="7" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
-    <cellStyle name="{Thousand}" xfId="8" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="{Z'0000(1 dec)}" xfId="9" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="{Z'0000(4 dec)}" xfId="10" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
-    <cellStyle name="0%" xfId="103" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
-    <cellStyle name="0.0%" xfId="104" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="0.00%" xfId="105" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
-    <cellStyle name="20% - Accent1" xfId="11" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
-    <cellStyle name="20% - Accent2" xfId="12" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
-    <cellStyle name="20% - Accent3" xfId="13" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="20% - Accent4" xfId="14" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
-    <cellStyle name="20% - Accent5" xfId="15" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="20% - Accent6" xfId="16" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
-    <cellStyle name="40% - Accent1" xfId="17" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
-    <cellStyle name="40% - Accent2" xfId="18" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
-    <cellStyle name="40% - Accent3" xfId="19" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
-    <cellStyle name="40% - Accent4" xfId="20" xr:uid="{00000000-0005-0000-0000-000033000000}"/>
-    <cellStyle name="40% - Accent5" xfId="21" xr:uid="{00000000-0005-0000-0000-000034000000}"/>
-    <cellStyle name="40% - Accent6" xfId="22" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
-    <cellStyle name="60% - Accent1" xfId="23" xr:uid="{00000000-0005-0000-0000-000036000000}"/>
-    <cellStyle name="60% - Accent2" xfId="24" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
-    <cellStyle name="60% - Accent3" xfId="25" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
-    <cellStyle name="60% - Accent4" xfId="26" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
-    <cellStyle name="60% - Accent5" xfId="27" xr:uid="{00000000-0005-0000-0000-00003A000000}"/>
-    <cellStyle name="60% - Accent6" xfId="28" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
-    <cellStyle name="Accent1" xfId="29" xr:uid="{00000000-0005-0000-0000-00003C000000}"/>
-    <cellStyle name="Accent2" xfId="30" xr:uid="{00000000-0005-0000-0000-00003D000000}"/>
-    <cellStyle name="Accent3" xfId="31" xr:uid="{00000000-0005-0000-0000-00003E000000}"/>
-    <cellStyle name="Accent4" xfId="32" xr:uid="{00000000-0005-0000-0000-00003F000000}"/>
-    <cellStyle name="Accent5" xfId="33" xr:uid="{00000000-0005-0000-0000-000040000000}"/>
-    <cellStyle name="Accent6" xfId="34" xr:uid="{00000000-0005-0000-0000-000041000000}"/>
-    <cellStyle name="Bad" xfId="35" xr:uid="{00000000-0005-0000-0000-000042000000}"/>
-    <cellStyle name="Black" xfId="36" xr:uid="{00000000-0005-0000-0000-000043000000}"/>
-    <cellStyle name="Border" xfId="37" xr:uid="{00000000-0005-0000-0000-000044000000}"/>
-    <cellStyle name="Calc Currency (0)" xfId="106" xr:uid="{00000000-0005-0000-0000-000045000000}"/>
-    <cellStyle name="Calculation" xfId="38" xr:uid="{00000000-0005-0000-0000-000046000000}"/>
-    <cellStyle name="Check Cell" xfId="39" xr:uid="{00000000-0005-0000-0000-000047000000}"/>
-    <cellStyle name="Col Heads" xfId="107" xr:uid="{00000000-0005-0000-0000-000048000000}"/>
-    <cellStyle name="Column_Title" xfId="108" xr:uid="{00000000-0005-0000-0000-000049000000}"/>
-    <cellStyle name="Comma  - Style1" xfId="109" xr:uid="{00000000-0005-0000-0000-00004A000000}"/>
-    <cellStyle name="Comma  - Style2" xfId="110" xr:uid="{00000000-0005-0000-0000-00004B000000}"/>
-    <cellStyle name="Comma  - Style3" xfId="111" xr:uid="{00000000-0005-0000-0000-00004C000000}"/>
-    <cellStyle name="Comma  - Style4" xfId="112" xr:uid="{00000000-0005-0000-0000-00004D000000}"/>
-    <cellStyle name="Comma  - Style5" xfId="113" xr:uid="{00000000-0005-0000-0000-00004E000000}"/>
-    <cellStyle name="Comma  - Style6" xfId="114" xr:uid="{00000000-0005-0000-0000-00004F000000}"/>
-    <cellStyle name="Comma  - Style7" xfId="115" xr:uid="{00000000-0005-0000-0000-000050000000}"/>
-    <cellStyle name="Comma  - Style8" xfId="116" xr:uid="{00000000-0005-0000-0000-000051000000}"/>
-    <cellStyle name="Comma [0]_ rislugp" xfId="117" xr:uid="{00000000-0005-0000-0000-000052000000}"/>
-    <cellStyle name="Comma,0" xfId="118" xr:uid="{00000000-0005-0000-0000-000053000000}"/>
-    <cellStyle name="Comma,1" xfId="119" xr:uid="{00000000-0005-0000-0000-000054000000}"/>
-    <cellStyle name="Comma,2" xfId="120" xr:uid="{00000000-0005-0000-0000-000055000000}"/>
-    <cellStyle name="Comma_ rislugp" xfId="121" xr:uid="{00000000-0005-0000-0000-000056000000}"/>
-    <cellStyle name="Currency [0]_ rislugp" xfId="122" xr:uid="{00000000-0005-0000-0000-000057000000}"/>
-    <cellStyle name="Currency,0" xfId="123" xr:uid="{00000000-0005-0000-0000-000058000000}"/>
-    <cellStyle name="Currency,2" xfId="124" xr:uid="{00000000-0005-0000-0000-000059000000}"/>
-    <cellStyle name="Currency_ rislugp" xfId="125" xr:uid="{00000000-0005-0000-0000-00005A000000}"/>
-    <cellStyle name="Dezimal [0]_laroux" xfId="40" xr:uid="{00000000-0005-0000-0000-00005B000000}"/>
-    <cellStyle name="Dezimal_laroux" xfId="41" xr:uid="{00000000-0005-0000-0000-00005C000000}"/>
-    <cellStyle name="entry" xfId="126" xr:uid="{00000000-0005-0000-0000-00005D000000}"/>
-    <cellStyle name="entry box" xfId="127" xr:uid="{00000000-0005-0000-0000-00005E000000}"/>
-    <cellStyle name="Euro" xfId="42" xr:uid="{00000000-0005-0000-0000-00005F000000}"/>
-    <cellStyle name="Explanatory Text" xfId="43" xr:uid="{00000000-0005-0000-0000-000060000000}"/>
-    <cellStyle name="Followed Hyperlink_AheadBehind.xls Chart 23" xfId="44" xr:uid="{00000000-0005-0000-0000-000061000000}"/>
-    <cellStyle name="Good" xfId="45" xr:uid="{00000000-0005-0000-0000-000062000000}"/>
-    <cellStyle name="Grey" xfId="46" xr:uid="{00000000-0005-0000-0000-000063000000}"/>
-    <cellStyle name="Header1" xfId="128" xr:uid="{00000000-0005-0000-0000-000064000000}"/>
-    <cellStyle name="Header2" xfId="129" xr:uid="{00000000-0005-0000-0000-000065000000}"/>
-    <cellStyle name="Heading" xfId="47" xr:uid="{00000000-0005-0000-0000-000066000000}"/>
-    <cellStyle name="Heading 1" xfId="48" xr:uid="{00000000-0005-0000-0000-000067000000}"/>
-    <cellStyle name="Heading 2" xfId="49" xr:uid="{00000000-0005-0000-0000-000068000000}"/>
-    <cellStyle name="Heading 3" xfId="50" xr:uid="{00000000-0005-0000-0000-000069000000}"/>
-    <cellStyle name="Heading 4" xfId="51" xr:uid="{00000000-0005-0000-0000-00006A000000}"/>
-    <cellStyle name="Hyperlink_AheadBehind.xls Chart 23" xfId="52" xr:uid="{00000000-0005-0000-0000-00006B000000}"/>
-    <cellStyle name="Input" xfId="53" xr:uid="{00000000-0005-0000-0000-00006C000000}"/>
-    <cellStyle name="Input [yellow]" xfId="54" xr:uid="{00000000-0005-0000-0000-00006D000000}"/>
-    <cellStyle name="left" xfId="130" xr:uid="{00000000-0005-0000-0000-00006E000000}"/>
-    <cellStyle name="Linked Cell" xfId="55" xr:uid="{00000000-0005-0000-0000-00006F000000}"/>
-    <cellStyle name="Millares [0]_laroux" xfId="131" xr:uid="{00000000-0005-0000-0000-000070000000}"/>
-    <cellStyle name="Millares_laroux" xfId="132" xr:uid="{00000000-0005-0000-0000-000071000000}"/>
-    <cellStyle name="Milliers [0]_laroux" xfId="56" xr:uid="{00000000-0005-0000-0000-000072000000}"/>
-    <cellStyle name="Milliers_laroux" xfId="57" xr:uid="{00000000-0005-0000-0000-000073000000}"/>
-    <cellStyle name="Moneda [0]_laroux" xfId="133" xr:uid="{00000000-0005-0000-0000-000074000000}"/>
-    <cellStyle name="Moneda_laroux" xfId="134" xr:uid="{00000000-0005-0000-0000-000075000000}"/>
-    <cellStyle name="Mon閠aire [0]_laroux" xfId="135" xr:uid="{00000000-0005-0000-0000-000076000000}"/>
-    <cellStyle name="Mon閠aire_laroux" xfId="136" xr:uid="{00000000-0005-0000-0000-000077000000}"/>
-    <cellStyle name="Neutral" xfId="58" xr:uid="{00000000-0005-0000-0000-000078000000}"/>
-    <cellStyle name="no dec" xfId="137" xr:uid="{00000000-0005-0000-0000-000079000000}"/>
-    <cellStyle name="Non défini" xfId="59" xr:uid="{00000000-0005-0000-0000-00007A000000}"/>
-    <cellStyle name="Normal - Style1" xfId="60" xr:uid="{00000000-0005-0000-0000-00007B000000}"/>
-    <cellStyle name="Normal_ rislugp" xfId="138" xr:uid="{00000000-0005-0000-0000-00007C000000}"/>
-    <cellStyle name="Normalny_Arkusz1" xfId="139" xr:uid="{00000000-0005-0000-0000-00007D000000}"/>
-    <cellStyle name="Note" xfId="61" xr:uid="{00000000-0005-0000-0000-00007E000000}"/>
-    <cellStyle name="Output" xfId="62" xr:uid="{00000000-0005-0000-0000-00007F000000}"/>
-    <cellStyle name="Percent (0)" xfId="63" xr:uid="{00000000-0005-0000-0000-000080000000}"/>
-    <cellStyle name="Percent [2]" xfId="64" xr:uid="{00000000-0005-0000-0000-000081000000}"/>
-    <cellStyle name="Prefilled" xfId="140" xr:uid="{00000000-0005-0000-0000-000082000000}"/>
-    <cellStyle name="price" xfId="141" xr:uid="{00000000-0005-0000-0000-000083000000}"/>
-    <cellStyle name="Red" xfId="65" xr:uid="{00000000-0005-0000-0000-000084000000}"/>
-    <cellStyle name="revised" xfId="142" xr:uid="{00000000-0005-0000-0000-000085000000}"/>
-    <cellStyle name="S4" xfId="143" xr:uid="{00000000-0005-0000-0000-000086000000}"/>
-    <cellStyle name="S5" xfId="144" xr:uid="{00000000-0005-0000-0000-000087000000}"/>
-    <cellStyle name="section" xfId="145" xr:uid="{00000000-0005-0000-0000-000088000000}"/>
-    <cellStyle name="style" xfId="146" xr:uid="{00000000-0005-0000-0000-000089000000}"/>
-    <cellStyle name="style1" xfId="147" xr:uid="{00000000-0005-0000-0000-00008A000000}"/>
-    <cellStyle name="style2" xfId="148" xr:uid="{00000000-0005-0000-0000-00008B000000}"/>
-    <cellStyle name="Tickmark" xfId="66" xr:uid="{00000000-0005-0000-0000-00008C000000}"/>
-    <cellStyle name="Title" xfId="67" xr:uid="{00000000-0005-0000-0000-00008D000000}"/>
-    <cellStyle name="Total" xfId="68" xr:uid="{00000000-0005-0000-0000-00008E000000}"/>
-    <cellStyle name="Warning Text" xfId="69" xr:uid="{00000000-0005-0000-0000-00008F000000}"/>
-    <cellStyle name="wrap" xfId="149" xr:uid="{00000000-0005-0000-0000-000090000000}"/>
-    <cellStyle name="パーセント_laroux" xfId="150" xr:uid="{00000000-0005-0000-0000-000091000000}"/>
-    <cellStyle name="標準_１１月価格表" xfId="151" xr:uid="{00000000-0005-0000-0000-000092000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规 2" xfId="71" xr:uid="{00000000-0005-0000-0000-000094000000}"/>
-    <cellStyle name="常规_Book1" xfId="70" xr:uid="{00000000-0005-0000-0000-000095000000}"/>
-    <cellStyle name="常规_WOOKSHEET2" xfId="73" xr:uid="{00000000-0005-0000-0000-000096000000}"/>
-    <cellStyle name="常规_制造费用" xfId="72" xr:uid="{00000000-0005-0000-0000-000097000000}"/>
-    <cellStyle name="超级链接_B4-1审计项目工时预算与控制表(集团)" xfId="152" xr:uid="{00000000-0005-0000-0000-000098000000}"/>
-    <cellStyle name="分级显示行_1_4附件二凯旋评估表" xfId="153" xr:uid="{00000000-0005-0000-0000-000099000000}"/>
-    <cellStyle name="桁区切り [0.00]_１１月価格表" xfId="154" xr:uid="{00000000-0005-0000-0000-00009A000000}"/>
-    <cellStyle name="桁区切り_１１月価格表" xfId="155" xr:uid="{00000000-0005-0000-0000-00009B000000}"/>
-    <cellStyle name="霓付 [0]_97MBO" xfId="156" xr:uid="{00000000-0005-0000-0000-00009C000000}"/>
-    <cellStyle name="霓付_97MBO" xfId="157" xr:uid="{00000000-0005-0000-0000-00009D000000}"/>
-    <cellStyle name="烹拳 [0]_97MBO" xfId="158" xr:uid="{00000000-0005-0000-0000-00009E000000}"/>
-    <cellStyle name="烹拳_97MBO" xfId="159" xr:uid="{00000000-0005-0000-0000-00009F000000}"/>
-    <cellStyle name="普通_ 白土" xfId="160" xr:uid="{00000000-0005-0000-0000-0000A0000000}"/>
-    <cellStyle name="千分位[0]_ 白土" xfId="161" xr:uid="{00000000-0005-0000-0000-0000A1000000}"/>
-    <cellStyle name="千分位_ 白土" xfId="162" xr:uid="{00000000-0005-0000-0000-0000A2000000}"/>
-    <cellStyle name="千位[0]_97汇总" xfId="163" xr:uid="{00000000-0005-0000-0000-0000A3000000}"/>
-    <cellStyle name="千位_97汇总" xfId="164" xr:uid="{00000000-0005-0000-0000-0000A4000000}"/>
-    <cellStyle name="钎霖_laroux" xfId="165" xr:uid="{00000000-0005-0000-0000-0000A5000000}"/>
-    <cellStyle name="通貨 [0.00]_１１月価格表" xfId="166" xr:uid="{00000000-0005-0000-0000-0000A6000000}"/>
-    <cellStyle name="通貨_１１月価格表" xfId="167" xr:uid="{00000000-0005-0000-0000-0000A7000000}"/>
-    <cellStyle name="样式 1" xfId="168" xr:uid="{00000000-0005-0000-0000-0000A8000000}"/>
-    <cellStyle name="콤마 [0]_BOILER-CO1" xfId="169" xr:uid="{00000000-0005-0000-0000-0000A9000000}"/>
-    <cellStyle name="콤마_BOILER-CO1" xfId="170" xr:uid="{00000000-0005-0000-0000-0000AA000000}"/>
-    <cellStyle name="통화 [0]_BOILER-CO1" xfId="171" xr:uid="{00000000-0005-0000-0000-0000AB000000}"/>
-    <cellStyle name="통화_BOILER-CO1" xfId="172" xr:uid="{00000000-0005-0000-0000-0000AC000000}"/>
-    <cellStyle name="표준_0N-HANDLING " xfId="173" xr:uid="{00000000-0005-0000-0000-0000AD000000}"/>
+    <cellStyle name="@_text" xfId="1"/>
+    <cellStyle name="{Comma [0]}" xfId="2"/>
+    <cellStyle name="{Comma}" xfId="3"/>
+    <cellStyle name="{Date}" xfId="4"/>
+    <cellStyle name="{Month}" xfId="5"/>
+    <cellStyle name="{Percent}" xfId="6"/>
+    <cellStyle name="{Thousand [0]}" xfId="7"/>
+    <cellStyle name="{Thousand}" xfId="8"/>
+    <cellStyle name="{Z'0000(1 dec)}" xfId="9"/>
+    <cellStyle name="{Z'0000(4 dec)}" xfId="10"/>
+    <cellStyle name="20% - Accent1" xfId="11"/>
+    <cellStyle name="20% - Accent2" xfId="12"/>
+    <cellStyle name="20% - Accent3" xfId="13"/>
+    <cellStyle name="20% - Accent4" xfId="14"/>
+    <cellStyle name="20% - Accent5" xfId="15"/>
+    <cellStyle name="20% - Accent6" xfId="16"/>
+    <cellStyle name="40% - Accent1" xfId="17"/>
+    <cellStyle name="40% - Accent2" xfId="18"/>
+    <cellStyle name="40% - Accent3" xfId="19"/>
+    <cellStyle name="40% - Accent4" xfId="20"/>
+    <cellStyle name="40% - Accent5" xfId="21"/>
+    <cellStyle name="40% - Accent6" xfId="22"/>
+    <cellStyle name="60% - Accent1" xfId="23"/>
+    <cellStyle name="60% - Accent2" xfId="24"/>
+    <cellStyle name="60% - Accent3" xfId="25"/>
+    <cellStyle name="60% - Accent4" xfId="26"/>
+    <cellStyle name="60% - Accent5" xfId="27"/>
+    <cellStyle name="60% - Accent6" xfId="28"/>
+    <cellStyle name="Accent1" xfId="29"/>
+    <cellStyle name="Accent2" xfId="30"/>
+    <cellStyle name="Accent3" xfId="31"/>
+    <cellStyle name="Accent4" xfId="32"/>
+    <cellStyle name="Accent5" xfId="33"/>
+    <cellStyle name="Accent6" xfId="34"/>
+    <cellStyle name="Bad" xfId="35"/>
+    <cellStyle name="Black" xfId="36"/>
+    <cellStyle name="Border" xfId="37"/>
+    <cellStyle name="Calculation" xfId="38"/>
+    <cellStyle name="Check Cell" xfId="39"/>
+    <cellStyle name="Dezimal [0]_laroux" xfId="40"/>
+    <cellStyle name="Dezimal_laroux" xfId="41"/>
+    <cellStyle name="Euro" xfId="42"/>
+    <cellStyle name="Explanatory Text" xfId="43"/>
+    <cellStyle name="Followed Hyperlink_AheadBehind.xls Chart 23" xfId="44"/>
+    <cellStyle name="Good" xfId="45"/>
+    <cellStyle name="Grey" xfId="46"/>
+    <cellStyle name="Heading" xfId="47"/>
+    <cellStyle name="Heading 1" xfId="48"/>
+    <cellStyle name="Heading 2" xfId="49"/>
+    <cellStyle name="Heading 3" xfId="50"/>
+    <cellStyle name="Heading 4" xfId="51"/>
+    <cellStyle name="Hyperlink_AheadBehind.xls Chart 23" xfId="52"/>
+    <cellStyle name="Input" xfId="53"/>
+    <cellStyle name="Input [yellow]" xfId="54"/>
+    <cellStyle name="Linked Cell" xfId="55"/>
+    <cellStyle name="Milliers [0]_laroux" xfId="56"/>
+    <cellStyle name="Milliers_laroux" xfId="57"/>
+    <cellStyle name="Neutral" xfId="58"/>
+    <cellStyle name="Non défini" xfId="59"/>
+    <cellStyle name="Normal - Style1" xfId="60"/>
+    <cellStyle name="Note" xfId="61"/>
+    <cellStyle name="Output" xfId="62"/>
+    <cellStyle name="Percent (0)" xfId="63"/>
+    <cellStyle name="Percent [2]" xfId="64"/>
+    <cellStyle name="Red" xfId="65"/>
+    <cellStyle name="Tickmark" xfId="66"/>
+    <cellStyle name="Title" xfId="67"/>
+    <cellStyle name="Total" xfId="68"/>
+    <cellStyle name="Warning Text" xfId="69"/>
+    <cellStyle name="常规_Book1" xfId="70"/>
+    <cellStyle name="常规 2" xfId="71"/>
+    <cellStyle name="常规_制造费用" xfId="72"/>
+    <cellStyle name="常规_WOOKSHEET2" xfId="73"/>
+    <cellStyle name="?" xfId="74"/>
+    <cellStyle name="?餡_x000c_k" xfId="75"/>
+    <cellStyle name="?餡_x000c_k?_x000d_^" xfId="76"/>
+    <cellStyle name="?餡_x000c_k?_x000d_^黇_x0001_??_x0007__x0001__x0001_" xfId="77"/>
+    <cellStyle name="_2005审计报表及附注-中国建材股份模板（房屋）" xfId="78"/>
+    <cellStyle name="_2006年年报审计PBC表-XXX" xfId="79"/>
+    <cellStyle name="_2006年年报审计填报资料" xfId="80"/>
+    <cellStyle name="_PBC审核提示" xfId="81"/>
+    <cellStyle name="_宝丽华房地产20051231" xfId="82"/>
+    <cellStyle name="_保证金-企业填写部分" xfId="83"/>
+    <cellStyle name="_北新房屋2004年审-刘" xfId="84"/>
+    <cellStyle name="_北新股份2005年审工作底稿" xfId="85"/>
+    <cellStyle name="_北新建材关连交易基础表051230（10－12月版）更新稿" xfId="86"/>
+    <cellStyle name="_北新建材-会计报表附注模版" xfId="87"/>
+    <cellStyle name="_北新龙之星2004年审工作底稿" xfId="88"/>
+    <cellStyle name="_北新物流2005底稿-刘" xfId="89"/>
+    <cellStyle name="_北新置换memo" xfId="90"/>
+    <cellStyle name="_存货结转测试" xfId="91"/>
+    <cellStyle name="_存货数量与明细05.12" xfId="92"/>
+    <cellStyle name="_动力厂2004年审工作底稿-刘" xfId="93"/>
+    <cellStyle name="_分工" xfId="94"/>
+    <cellStyle name="_工程施工项目现场审计提示" xfId="95"/>
+    <cellStyle name="_关联交易" xfId="96"/>
+    <cellStyle name="_关联交易、往来统计表" xfId="97"/>
+    <cellStyle name="_科目核对表" xfId="98"/>
+    <cellStyle name="_母PL" xfId="99"/>
+    <cellStyle name="_人员分工备忘录" xfId="100"/>
+    <cellStyle name="_审计所需资料清单－子公司" xfId="101"/>
+    <cellStyle name="_长期借款－江阴" xfId="102"/>
+    <cellStyle name="0%" xfId="103"/>
+    <cellStyle name="0.0%" xfId="104"/>
+    <cellStyle name="0.00%" xfId="105"/>
+    <cellStyle name="Calc Currency (0)" xfId="106"/>
+    <cellStyle name="Col Heads" xfId="107"/>
+    <cellStyle name="Column_Title" xfId="108"/>
+    <cellStyle name="Comma  - Style1" xfId="109"/>
+    <cellStyle name="Comma  - Style2" xfId="110"/>
+    <cellStyle name="Comma  - Style3" xfId="111"/>
+    <cellStyle name="Comma  - Style4" xfId="112"/>
+    <cellStyle name="Comma  - Style5" xfId="113"/>
+    <cellStyle name="Comma  - Style6" xfId="114"/>
+    <cellStyle name="Comma  - Style7" xfId="115"/>
+    <cellStyle name="Comma  - Style8" xfId="116"/>
+    <cellStyle name="Comma [0]_ rislugp" xfId="117"/>
+    <cellStyle name="Comma,0" xfId="118"/>
+    <cellStyle name="Comma,1" xfId="119"/>
+    <cellStyle name="Comma,2" xfId="120"/>
+    <cellStyle name="Comma_ rislugp" xfId="121"/>
+    <cellStyle name="Currency [0]_ rislugp" xfId="122"/>
+    <cellStyle name="Currency,0" xfId="123"/>
+    <cellStyle name="Currency,2" xfId="124"/>
+    <cellStyle name="Currency_ rislugp" xfId="125"/>
+    <cellStyle name="entry" xfId="126"/>
+    <cellStyle name="entry box" xfId="127"/>
+    <cellStyle name="Header1" xfId="128"/>
+    <cellStyle name="Header2" xfId="129"/>
+    <cellStyle name="left" xfId="130"/>
+    <cellStyle name="Millares [0]_laroux" xfId="131"/>
+    <cellStyle name="Millares_laroux" xfId="132"/>
+    <cellStyle name="Moneda [0]_laroux" xfId="133"/>
+    <cellStyle name="Moneda_laroux" xfId="134"/>
+    <cellStyle name="Mon閠aire [0]_laroux" xfId="135"/>
+    <cellStyle name="Mon閠aire_laroux" xfId="136"/>
+    <cellStyle name="no dec" xfId="137"/>
+    <cellStyle name="Normal_ rislugp" xfId="138"/>
+    <cellStyle name="Normalny_Arkusz1" xfId="139"/>
+    <cellStyle name="Prefilled" xfId="140"/>
+    <cellStyle name="price" xfId="141"/>
+    <cellStyle name="revised" xfId="142"/>
+    <cellStyle name="S4" xfId="143"/>
+    <cellStyle name="S5" xfId="144"/>
+    <cellStyle name="section" xfId="145"/>
+    <cellStyle name="style" xfId="146"/>
+    <cellStyle name="style1" xfId="147"/>
+    <cellStyle name="style2" xfId="148"/>
+    <cellStyle name="wrap" xfId="149"/>
+    <cellStyle name="パーセント_laroux" xfId="150"/>
+    <cellStyle name="標準_１１月価格表" xfId="151"/>
+    <cellStyle name="超级链接_B4-1审计项目工时预算与控制表(集团)" xfId="152"/>
+    <cellStyle name="分级显示行_1_4附件二凯旋评估表" xfId="153"/>
+    <cellStyle name="桁区切り [0.00]_１１月価格表" xfId="154"/>
+    <cellStyle name="桁区切り_１１月価格表" xfId="155"/>
+    <cellStyle name="霓付 [0]_97MBO" xfId="156"/>
+    <cellStyle name="霓付_97MBO" xfId="157"/>
+    <cellStyle name="烹拳 [0]_97MBO" xfId="158"/>
+    <cellStyle name="烹拳_97MBO" xfId="159"/>
+    <cellStyle name="普通_ 白土" xfId="160"/>
+    <cellStyle name="千分位[0]_ 白土" xfId="161"/>
+    <cellStyle name="千分位_ 白土" xfId="162"/>
+    <cellStyle name="千位[0]_97汇总" xfId="163"/>
+    <cellStyle name="千位_97汇总" xfId="164"/>
+    <cellStyle name="钎霖_laroux" xfId="165"/>
+    <cellStyle name="通貨 [0.00]_１１月価格表" xfId="166"/>
+    <cellStyle name="通貨_１１月価格表" xfId="167"/>
+    <cellStyle name="样式 1" xfId="168"/>
+    <cellStyle name="콤마 [0]_BOILER-CO1" xfId="169"/>
+    <cellStyle name="콤마_BOILER-CO1" xfId="170"/>
+    <cellStyle name="통화 [0]_BOILER-CO1" xfId="171"/>
+    <cellStyle name="통화_BOILER-CO1" xfId="172"/>
+    <cellStyle name="표준_0N-HANDLING " xfId="173"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="G9-1"/>
@@ -1985,7 +1901,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink10.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="分工"/>
@@ -2747,7 +2663,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink11.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="分工"/>
@@ -3587,7 +3503,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink12.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="分工"/>
@@ -4367,7 +4283,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink13.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="索引"/>
@@ -4394,7 +4310,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink14.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="G9-1"/>
@@ -4582,7 +4498,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink15.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="徐"/>
@@ -4977,7 +4893,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="1"/>
@@ -5783,7 +5699,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="徐"/>
@@ -5800,7 +5716,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="1"/>
@@ -5866,7 +5782,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="1"/>
@@ -6565,7 +6481,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Breakdown"/>
@@ -8852,7 +8768,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink7.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="breakdown"/>
@@ -10655,7 +10571,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink8.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="分工"/>
@@ -11393,7 +11309,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink9.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="1"/>
@@ -12476,286 +12392,400 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="20.100000000000001" customHeight="1"/>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="20.1" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4" style="13" customWidth="1"/>
-    <col min="2" max="4" width="23.59765625" style="13" customWidth="1"/>
-    <col min="5" max="5" width="5.19921875" style="13" customWidth="1"/>
-    <col min="6" max="6" width="6.5" style="13" customWidth="1"/>
-    <col min="7" max="7" width="7.3984375" style="13" customWidth="1"/>
-    <col min="8" max="8" width="6.69921875" style="13" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="13"/>
+    <col width="4" customWidth="1" style="13" min="1" max="1"/>
+    <col width="23.59765625" customWidth="1" style="13" min="2" max="4"/>
+    <col width="5.19921875" customWidth="1" style="13" min="5" max="5"/>
+    <col width="6.5" customWidth="1" style="13" min="6" max="6"/>
+    <col width="7.3984375" customWidth="1" style="13" min="7" max="7"/>
+    <col width="6.69921875" customWidth="1" style="13" min="8" max="8"/>
+    <col width="9" customWidth="1" style="13" min="9" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="4" customFormat="1" ht="19.95" customHeight="1">
-      <c r="A1" s="2"/>
-      <c r="B1" s="18" t="s">
-        <v>16</v>
+    <row r="1" ht="19.95" customFormat="1" customHeight="1" s="4">
+      <c r="A1" s="2" t="n"/>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>致同会计师事务所</t>
+        </is>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="3"/>
+      <c r="I1" s="3" t="n"/>
     </row>
-    <row r="2" spans="1:9" s="4" customFormat="1" ht="19.95" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="19" t="s">
-        <v>30</v>
+    <row r="2" ht="19.95" customFormat="1" customHeight="1" s="4">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>重大事项概要程序表</t>
+        </is>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="3"/>
+      <c r="I2" s="3" t="n"/>
     </row>
-    <row r="3" spans="1:9" s="9" customFormat="1" ht="19.95" customHeight="1">
-      <c r="A3" s="5" t="s">
-        <v>17</v>
+    <row r="3" ht="19.95" customFormat="1" customHeight="1" s="9">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>客户名称：</t>
+        </is>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="6" t="s">
-        <v>18</v>
+      <c r="B3" s="0" t="n"/>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>编制人：</t>
+        </is>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>31</v>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>日期：</t>
+        </is>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="6" t="s">
-        <v>34</v>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>索引号：</t>
+        </is>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>23</v>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>A17</t>
+        </is>
       </c>
-      <c r="I3" s="8"/>
+      <c r="I3" s="8" t="n"/>
     </row>
-    <row r="4" spans="1:9" s="9" customFormat="1" ht="19.95" customHeight="1">
-      <c r="A4" s="6" t="s">
-        <v>35</v>
+    <row r="4" ht="19.95" customFormat="1" customHeight="1" s="9">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>会计期间：201X年度</t>
+        </is>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6" t="s">
-        <v>36</v>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>复核人：</t>
+        </is>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>31</v>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>日期：</t>
+        </is>
       </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="6" t="s">
-        <v>37</v>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>页  次：</t>
+        </is>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="8"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="8" t="n"/>
     </row>
-    <row r="5" spans="1:9" ht="29.4" customHeight="1">
-      <c r="A5" s="10" t="s">
-        <v>19</v>
+    <row r="5" ht="29.4" customHeight="1" s="20">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>29</v>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>程序</t>
+        </is>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="12" t="s">
-        <v>20</v>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>是否适用</t>
+        </is>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>38</v>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>执行人</t>
+        </is>
       </c>
-      <c r="G5" s="12" t="s">
-        <v>21</v>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>执行情况说明</t>
+        </is>
       </c>
-      <c r="H5" s="12" t="s">
-        <v>22</v>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>索引号</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="19.95" customHeight="1">
-      <c r="A6" s="14">
+    <row r="6" ht="19.95" customHeight="1" s="20">
+      <c r="A6" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>32</v>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>汇总重大职业判断以及需合伙人关注事项，详细说明审计程序执行情况。</t>
+        </is>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="16" t="s">
-        <v>24</v>
+      <c r="C6" s="23" t="n"/>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>A17-1</t>
+        </is>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="19.95" customHeight="1">
-      <c r="A7" s="14">
+    <row r="7" ht="19.95" customHeight="1" s="20">
+      <c r="A7" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>39</v>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>对于咨询的重大会计或审计事项咨询，确定咨询报告是否包括在审计工作底稿中；如有咨询结论，同步记录执行情况（A17-3-1）。</t>
+        </is>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="16" t="s">
-        <v>25</v>
+      <c r="C7" s="23" t="n"/>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>A17-3</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="29.4" customHeight="1">
-      <c r="A8" s="14">
+    <row r="8" ht="29.4" customHeight="1" s="20">
+      <c r="A8" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>40</v>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>对于项目组的专业意见分歧，确认已经得到解决，并将解决方式、解决过程、解决结论等记录于工作底稿。</t>
+        </is>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="16" t="s">
-        <v>26</v>
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>A17-4</t>
+        </is>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="139.19999999999999" customHeight="1">
-      <c r="A9" s="14">
+    <row r="9" ht="139.2" customHeight="1" s="20">
+      <c r="A9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>33</v>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>确定在审计过程中识别的重大职业判断以及需合伙人关注事项是否包括在重大事项概要汇总表中，并完成关键审计事项（KAM）专项底稿（上市实体或法规要求披露 KAM 时适用）：
+（1）引起特别风险的事项；
+（2）已更正或未更正的错报；
+（3）值得关注的缺陷和其他控制缺陷；
+（4）重大职业判断；
+（5）业务咨询和意见分歧；
+（6）导致注册会计师难以实施必要审计程序的情形；
+（7）可能导致出具非无保留意见审计报告的事项；
+（8）独立性威胁或利益冲突。</t>
+        </is>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="16" t="s">
-        <v>27</v>
+      <c r="C9" s="23" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>A17-2-1</t>
+        </is>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="19.95" customHeight="1">
-      <c r="A10" s="14">
+    <row r="10" ht="19.95" customHeight="1" s="20">
+      <c r="A10" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>41</v>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>召开项目组总结会并将会议纪要记录于工作底稿。</t>
+        </is>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="16" t="s">
-        <v>28</v>
+      <c r="C10" s="23" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="17" t="n"/>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>A17-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>完成审计工作完成核对表（按业务类型选用 A17-5-1~5-5：A 类财报必做 A17-5-1；整合审计追加 A17-5-2；IPO 追加 A17-5-3；新三板追加 A17-5-4；函证程序推荐 A17-5-5），确认所有「否」项已处理完毕。</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>A17-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>审计项目团队成员签署独立性声明书（完成阶段）；专业技术委员会审核委员使用 A17-7A。签署日期不晚于审计报告日。</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>A17-7</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B7:D7"/>
     <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B9:D9"/>
   </mergeCells>
-  <phoneticPr fontId="36" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E10" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation sqref="E6:E10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"是,否"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.98425196850393704" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="77" fitToHeight="100" orientation="portrait" blackAndWhite="1" cellComments="atEnd" r:id="rId1"/>
-  <headerFooter alignWithMargins="0"/>
+  <pageMargins left="0.984251968503937" right="0.7480314960629921" top="0.984251968503937" bottom="0.984251968503937" header="0.5118110236220472" footer="0.5118110236220472"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="77" fitToHeight="100" blackAndWhite="1" cellComments="atEnd"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6"/>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>0</v>
+    <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>Custom 1</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>2</v>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>Custom 2</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>4</v>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Custom 3</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>6</v>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Custom 4</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>8</v>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Custom 5</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>10</v>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
       </c>
-      <c r="B6" t="s">
-        <v>11</v>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Custom 6</t>
+        </is>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>12</v>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
       </c>
-      <c r="B7" t="s">
-        <v>13</v>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Custom 7</t>
+        </is>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>14</v>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
       </c>
-      <c r="B8" t="s">
-        <v>15</v>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Custom 8</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>